<commit_message>
Add cross-sheet navigation and reading path for v2 docs
Co-authored-by: nguyenpr9 <nguyenpr9@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Basic Design v2.xlsx
+++ b/Basic Design v2.xlsx
@@ -8,34 +8,36 @@
   </bookViews>
   <sheets>
     <sheet name="00_ReadMe_Visual" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Architecture_Flow_v2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="KPI_Story_Chart" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dashboard_Wireframe_v2" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Header" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="History" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Overview" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Modules" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Dashboards" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="KPI" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="DataModel" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="SourceMapping" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="DAXLogic" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="BusinessRules" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="RLS" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="SignOff_v2" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="01_Reading_Path_v2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Architecture_Flow_v2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="KPI_Story_Chart" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dashboard_Wireframe_v2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Header" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="History" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Overview" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Modules" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Dashboards" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="KPI" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="DataModel" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="SourceMapping" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DAXLogic" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="BusinessRules" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="RLS" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="SignOff_v2" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Header'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'History'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Overview'!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Modules'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Dashboards'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'KPI'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'DataModel'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'SourceMapping'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'DAXLogic'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'BusinessRules'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'RLS'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Reading_Path_v2'!$A$6:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Header'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'History'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Overview'!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Modules'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Dashboards'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'KPI'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'DataModel'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'SourceMapping'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'DAXLogic'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'BusinessRules'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'RLS'!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,7 +46,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,6 +81,16 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="13">
@@ -247,10 +259,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -326,9 +339,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -1279,7 +1299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F14"/>
+  <dimension ref="B2:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1383,18 +1403,369 @@
       <c r="E14" s="27" t="n"/>
       <c r="F14" s="28" t="n"/>
     </row>
+    <row r="17">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Quick Links - Bắt đầu đọc từ đây</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="9" t="n"/>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Mục tiêu</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>00_ReadMe_Visual</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Nắm cấu trúc tài liệu và legend màu</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="32" t="inlineStr">
+        <is>
+          <t>Architecture_Flow_v2</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu kiến trúc end-to-end từ source đến report</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="32" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu tầng dữ liệu, flow và quy tắc triển khai mức cao</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" s="32" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu từng subject area và người dùng chính</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" s="32" t="inlineStr">
+        <is>
+          <t>Dashboards</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu dashboard mục tiêu và insight kỳ vọng</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" s="32" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu định nghĩa KPI và ngưỡng cảnh báo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" s="32" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu fact/dim và khóa liên kết chính</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" s="32" t="inlineStr">
+        <is>
+          <t>SourceMapping</t>
+        </is>
+      </c>
+      <c r="D26" s="23" t="inlineStr">
+        <is>
+          <t>Map chi tiết từ SQL Server sang Power BI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="B2:F3"/>
+    <mergeCell ref="B17:G17"/>
     <mergeCell ref="D5:F9"/>
-    <mergeCell ref="B2:F3"/>
     <mergeCell ref="B11:F14"/>
     <mergeCell ref="B5:C9"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId8"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="43" customWidth="1" min="5" max="5"/>
+    <col width="78" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tên Dashboard</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mục tiêu phân tích</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Người sử dụng</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Bố cục chi tiết</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Mockup ASCII</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Insight chính</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Executive Portfolio Overview</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi tình trạng toàn bộ danh mục dự án ở cấp điều hành.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CEO, COO, PMO Director</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Top: 6 KPI card. Left: Column Actual vs Budget. Right: Line Cashflow theo tháng. Bottom: Matrix top overspend.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[KPI x6]
+[Column Actual vs Budget] [Line Cashflow]
+[Matrix Overspend]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Nhận diện sớm dự án vượt ngân sách và chậm tiến độ để tái phân bổ nguồn lực.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Material Consumption Control</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Giám sát tiêu thụ vật tư theo nhóm vật liệu, dự án và nhà thầu.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Project Manager, Site Engineer</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Top-left KPI card; top-right donut vật tư; middle stacked column theo dự án; bottom bảng giao dịch chi tiết.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>[KPI]
+[Donut Material Mix] [Stacked Column]
+[Transaction Table]</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Phát hiện nhóm vật tư gây overuse và điểm nóng hao hụt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Cost vs Budget Deep Dive</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Phân tích sai lệch ngân sách theo category và nhà thầu.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Finance Controller, PM</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Top KPI; left waterfall variance bridge; right bar theo cost category; bottom matrix drilldown.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>[KPI]
+[Waterfall] [Bar]
+[Matrix Drilldown]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Khoanh vùng nguyên nhân vượt chi phí để hành động cắt giảm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Progress &amp; Delay Risk</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi tiến độ và cảnh báo rủi ro trễ milestone.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Planning Engineer, PM</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Top KPI; left line planned vs actual; right heatmap delay; bottom table milestone.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>[KPI]
+[Line Planned vs Actual] [Heatmap]
+[Milestone Table]</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Ưu tiên xử lý work package có delay &gt; 7 ngày hoặc SPI &lt; 0.95.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1788,7 +2159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2182,7 +2553,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2761,7 +3132,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2948,7 +3319,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3213,7 +3584,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3370,7 +3741,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3573,6 +3944,549 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BASIC DESIGN - RECOMMENDED READING PATH</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Đọc theo thứ tự từ trên xuống. Cột "Liên kết sheet" có hyperlink để nhảy trực tiếp tới sheet tương ứng.</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
+      <c r="G3" s="15" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="n"/>
+      <c r="B4" s="15" t="n"/>
+      <c r="C4" s="15" t="n"/>
+      <c r="D4" s="15" t="n"/>
+      <c r="E4" s="15" t="n"/>
+      <c r="F4" s="15" t="n"/>
+      <c r="G4" s="15" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Liên kết sheet</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Mục tiêu đọc</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Input nhận từ</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Output chuyển tới</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Persona chính</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Kết quả kỳ vọng</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>00_ReadMe_Visual</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Nắm cấu trúc tài liệu và legend màu</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Architecture_Flow_v2</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>Biết bức tranh tổng thể</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Architecture_Flow_v2</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu kiến trúc end-to-end từ source đến report</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>ReadMe</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>Stakeholder + Architect</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>Thống nhất scope kỹ thuật</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu tầng dữ liệu, flow và quy tắc triển khai mức cao</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>PMO + Business</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>Khóa phạm vi nghiệp vụ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu từng subject area và người dùng chính</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>Dashboards</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>Business Owner</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>Chốt module ưu tiên</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>Dashboards</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu dashboard mục tiêu và insight kỳ vọng</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>Sponsor + BI Lead</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="inlineStr">
+        <is>
+          <t>Chốt hướng phân tích</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="32" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu định nghĩa KPI và ngưỡng cảnh báo</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>Dashboards</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>Business + Data</t>
+        </is>
+      </c>
+      <c r="G12" s="23" t="inlineStr">
+        <is>
+          <t>Chốt logic đo lường</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu fact/dim và khóa liên kết chính</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>SourceMapping</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="G13" s="23" t="inlineStr">
+        <is>
+          <t>Chốt khung semantic model</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>SourceMapping</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>Map chi tiết từ SQL Server sang Power BI</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>DAXLogic</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>ETL Dev</t>
+        </is>
+      </c>
+      <c r="G14" s="23" t="inlineStr">
+        <is>
+          <t>Triển khai pipeline ETL</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="31" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t>DAXLogic</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu công thức measure chính</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>KPI + Model</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Power BI Dev</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="inlineStr">
+        <is>
+          <t>Triển khai semantic logic</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu luật nghiệp vụ và ngoại lệ</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>DAX + Mapping</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>RLS</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>Business + QA</t>
+        </is>
+      </c>
+      <c r="G16" s="23" t="inlineStr">
+        <is>
+          <t>Chốt test case nghiệp vụ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="31" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>RLS</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu role và phân quyền dữ liệu</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>SignOff_v2</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Security + PM</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="inlineStr">
+        <is>
+          <t>Sẵn sàng UAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>SignOff_v2</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Ký xác nhận liên phòng ban</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>All previous</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>Go-live prep</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>PMO + Sponsor</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>Đủ điều kiện triển khai</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:G18"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:G4"/>
+    <mergeCell ref="A1:G2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId12"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3908,7 +4822,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4305,7 +5219,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4850,7 +5764,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4943,7 +5857,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>v2.0 - Basic Design (Visual Enhanced)</t>
+          <t>v2.1 - Basic Design (Visual + Navigation Linked)</t>
         </is>
       </c>
     </row>
@@ -4977,13 +5891,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5124,23 +6038,49 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>v2.1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Senior BI Solution Architect</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Bổ sung Reading Path + hyperlink giữa Overview và các sheet để điều hướng theo thứ tự đọc.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5237,13 +6177,434 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>NAVIGATION FROM OVERVIEW</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="1" t="n"/>
+      <c r="D9" s="1" t="n"/>
+      <c r="E9" s="1" t="n"/>
+      <c r="F9" s="1" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Đi tới sheet</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Đọc để làm gì</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Ai nên đọc</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>00_ReadMe_Visual</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Nắm cấu trúc tài liệu và legend màu</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>Architecture_Flow_v2</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="32" t="inlineStr">
+        <is>
+          <t>Architecture_Flow_v2</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu kiến trúc end-to-end từ source đến report</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>ReadMe</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>Stakeholder + Architect</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu tầng dữ liệu, flow và quy tắc triển khai mức cao</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>PMO + Business</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu từng subject area và người dùng chính</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>Overview</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>Dashboards</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>Business Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t>Dashboards</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu dashboard mục tiêu và insight kỳ vọng</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Sponsor + BI Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu định nghĩa KPI và ngưỡng cảnh báo</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>Dashboards</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>Business + Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu fact/dim và khóa liên kết chính</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>SourceMapping</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>SourceMapping</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>Map chi tiết từ SQL Server sang Power BI</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>DataModel</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>DAXLogic</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>ETL Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="31" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>DAXLogic</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu công thức measure chính</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>KPI + Model</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>Power BI Dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu luật nghiệp vụ và ngoại lệ</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>DAX + Mapping</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>RLS</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>Business + QA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="n">
+        <v>11</v>
+      </c>
+      <c r="B21" s="32" t="inlineStr">
+        <is>
+          <t>RLS</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>Hiểu role và phân quyền dữ liệu</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>BusinessRules</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="inlineStr">
+        <is>
+          <t>SignOff_v2</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>Security + PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="n">
+        <v>12</v>
+      </c>
+      <c r="B22" s="32" t="inlineStr">
+        <is>
+          <t>SignOff_v2</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="inlineStr">
+        <is>
+          <t>Ký xác nhận liên phòng ban</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>All previous</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="inlineStr">
+        <is>
+          <t>Go-live prep</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="inlineStr">
+        <is>
+          <t>PMO + Sponsor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A9:F9"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId12"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5425,195 +6786,4 @@
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="80" customWidth="1" min="4" max="4"/>
-    <col width="43" customWidth="1" min="5" max="5"/>
-    <col width="78" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Tên Dashboard</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Mục tiêu phân tích</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Người sử dụng</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Bố cục chi tiết</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Mockup ASCII</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Insight chính</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Executive Portfolio Overview</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Theo dõi tình trạng toàn bộ danh mục dự án ở cấp điều hành.</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>CEO, COO, PMO Director</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Top: 6 KPI card. Left: Column Actual vs Budget. Right: Line Cashflow theo tháng. Bottom: Matrix top overspend.</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>[KPI x6]
-[Column Actual vs Budget] [Line Cashflow]
-[Matrix Overspend]</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Nhận diện sớm dự án vượt ngân sách và chậm tiến độ để tái phân bổ nguồn lực.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Material Consumption Control</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Giám sát tiêu thụ vật tư theo nhóm vật liệu, dự án và nhà thầu.</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Project Manager, Site Engineer</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Top-left KPI card; top-right donut vật tư; middle stacked column theo dự án; bottom bảng giao dịch chi tiết.</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>[KPI]
-[Donut Material Mix] [Stacked Column]
-[Transaction Table]</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Phát hiện nhóm vật tư gây overuse và điểm nóng hao hụt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Cost vs Budget Deep Dive</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Phân tích sai lệch ngân sách theo category và nhà thầu.</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Finance Controller, PM</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Top KPI; left waterfall variance bridge; right bar theo cost category; bottom matrix drilldown.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>[KPI]
-[Waterfall] [Bar]
-[Matrix Drilldown]</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Khoanh vùng nguyên nhân vượt chi phí để hành động cắt giảm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Progress &amp; Delay Risk</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Theo dõi tiến độ và cảnh báo rủi ro trễ milestone.</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Planning Engineer, PM</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Top KPI; left line planned vs actual; right heatmap delay; bottom table milestone.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>[KPI]
-[Line Planned vs Actual] [Heatmap]
-[Milestone Table]</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Ưu tiên xử lý work package có delay &gt; 7 ngày hoặc SPI &lt; 0.95.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>